<commit_message>
zpl code for pack id changed accrding to new label (unified), app.py updated acording to the need
</commit_message>
<xml_diff>
--- a/models/hv/data/pack_id_scan_log.xlsx
+++ b/models/hv/data/pack_id_scan_log.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3036" yWindow="2340" windowWidth="11268" windowHeight="9900" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Pack ID" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pack ID" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1071,6 +1071,366 @@
         </is>
       </c>
     </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>9:16:27 AM</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>ABA51202605281A00111</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281A00111</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>10:10:16 AM</t>
+        </is>
+      </c>
+      <c r="D22" s="7" t="inlineStr">
+        <is>
+          <t>ABA51202605281A00001</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>12P</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
+        <is>
+          <t>VX156080:ABA51202605281A00001</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>10:10:33 AM</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>ABA51202605281A00002</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>16P</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>VX156070:ABA51202605281A00002</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>10:12:14 AM</t>
+        </is>
+      </c>
+      <c r="D24" s="7" t="inlineStr">
+        <is>
+          <t>ABA51202605281A00003</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F24" s="7" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281A00003</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>10:12:33 AM</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>ABA51202605281A00004</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>27P</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>VX155800:ABA51202605281A00004</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>12:51:14 PM</t>
+        </is>
+      </c>
+      <c r="D26" s="7" t="inlineStr">
+        <is>
+          <t>ABA51202605281A00001</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>12P</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>VX156080:ABA51202605281A00001</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>1:03:22 PM</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>ABA51202605281A00001</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>12P</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>VX156080:ABA51202605281A00001</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>1:03:57 PM</t>
+        </is>
+      </c>
+      <c r="D28" s="7" t="inlineStr">
+        <is>
+          <t>ABA51202605281A00002</t>
+        </is>
+      </c>
+      <c r="E28" s="6" t="inlineStr">
+        <is>
+          <t>16P</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>VX156070:ABA51202605281A00002</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>1:04:09 PM</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>ABA51202605281A00003</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281A00003</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>1:04:21 PM</t>
+        </is>
+      </c>
+      <c r="D30" s="7" t="inlineStr">
+        <is>
+          <t>ABA51202605281A00004</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
+        <is>
+          <t>27P</t>
+        </is>
+      </c>
+      <c r="F30" s="7" t="inlineStr">
+        <is>
+          <t>VX155800:ABA51202605281A00004</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>1:07:38 PM</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>ABA51202605281A00003</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281A00003</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>21 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>1:49:02 PM</t>
+        </is>
+      </c>
+      <c r="D32" s="7" t="inlineStr">
+        <is>
+          <t>ABA51202609211A00009</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F32" s="7" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202609211A00009</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
serial count changed to 6 digits, group to 1-3
</commit_message>
<xml_diff>
--- a/models/hv/data/pack_id_scan_log.xlsx
+++ b/models/hv/data/pack_id_scan_log.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1701,6 +1701,36 @@
         </is>
       </c>
     </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="6" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>3:29:39 PM</t>
+        </is>
+      </c>
+      <c r="D42" s="7" t="inlineStr">
+        <is>
+          <t>ABA51202605281A123456</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F42" s="7" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281A123456</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
part number updated for bak-VQ... and for Ten Power-VX... and accepts only respective modules ids
</commit_message>
<xml_diff>
--- a/models/hv/data/pack_id_scan_log.xlsx
+++ b/models/hv/data/pack_id_scan_log.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F42"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1731,6 +1731,336 @@
         </is>
       </c>
     </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="4" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>23 Aug 2026</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>3:41:08 PM</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>ABA31202608231A00289</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>12P</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="inlineStr">
+        <is>
+          <t>VQ150000:ABA31202608231A00289</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="6" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>23 Aug 2026</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>3:43:01 PM</t>
+        </is>
+      </c>
+      <c r="D44" s="7" t="inlineStr">
+        <is>
+          <t>ABA31202608231A00289</t>
+        </is>
+      </c>
+      <c r="E44" s="6" t="inlineStr">
+        <is>
+          <t>12P</t>
+        </is>
+      </c>
+      <c r="F44" s="7" t="inlineStr">
+        <is>
+          <t>VQ150000:ABA31202608231A00289</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="4" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>23 Aug 2026</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>3:44:42 PM</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>ABA31202608231A00289</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>12P</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>VQ150000:ABA31202608231A00289</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="6" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>25 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>3:45:00 PM</t>
+        </is>
+      </c>
+      <c r="D46" s="7" t="inlineStr">
+        <is>
+          <t>ABA41202609251A00296</t>
+        </is>
+      </c>
+      <c r="E46" s="6" t="inlineStr">
+        <is>
+          <t>16P</t>
+        </is>
+      </c>
+      <c r="F46" s="7" t="inlineStr">
+        <is>
+          <t>VQ150010:ABA41202609251A00296</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="4" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>25 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>3:45:13 PM</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>ABA51202609251A00298</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr">
+        <is>
+          <t>VQ150020:ABA51202609251A00298</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="6" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>24 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>3:45:26 PM</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="inlineStr">
+        <is>
+          <t>ABA61202609241A00291</t>
+        </is>
+      </c>
+      <c r="E48" s="6" t="inlineStr">
+        <is>
+          <t>27P</t>
+        </is>
+      </c>
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t>VQ150030:ABA61202609241A00291</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="18" customHeight="1">
+      <c r="A49" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>23 Aug 2026</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>5:17:38 PM</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>ABA31202608231A00289</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>12P</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>VQ150000:ABA31202608231A00289</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="18" customHeight="1">
+      <c r="A50" s="6" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>7:15:33 PM</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>ABA51202605281A00111</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F50" s="7" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281A00111</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="18" customHeight="1">
+      <c r="A51" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>25 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>7:57:34 PM</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>ABA41202609251A00296</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>16P</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>VQ150010:ABA41202609251A00296</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="18" customHeight="1">
+      <c r="A52" s="6" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>23 Aug 2026</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>7:58:01 PM</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="inlineStr">
+        <is>
+          <t>ABA31202608231A00289</t>
+        </is>
+      </c>
+      <c r="E52" s="6" t="inlineStr">
+        <is>
+          <t>12P</t>
+        </is>
+      </c>
+      <c r="F52" s="7" t="inlineStr">
+        <is>
+          <t>VQ150000:ABA31202608231A00289</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="18" customHeight="1">
+      <c r="A53" s="4" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>7:58:29 PM</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>ABA51202605281A00111</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281A00111</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
serial number (shift), dummy id (select), zpl (mfg_year) are unaltered
</commit_message>
<xml_diff>
--- a/models/hv/data/pack_id_scan_log.xlsx
+++ b/models/hv/data/pack_id_scan_log.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2061,6 +2061,96 @@
         </is>
       </c>
     </row>
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="6" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>11:03:03 AM</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>ABA51202605281A00111</t>
+        </is>
+      </c>
+      <c r="E54" s="6" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F54" s="7" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281A00111</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="18" customHeight="1">
+      <c r="A55" s="4" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>11:03:57 AM</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>ABA51202605281A00111</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281A00111</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="18" customHeight="1">
+      <c r="A56" s="6" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>11:10:00 AM</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="inlineStr">
+        <is>
+          <t>ABA51202605281A00111</t>
+        </is>
+      </c>
+      <c r="E56" s="6" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F56" s="7" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281A00111</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
mfg format changed for fg sticker label, made in india image to zpl changed
</commit_message>
<xml_diff>
--- a/models/hv/data/pack_id_scan_log.xlsx
+++ b/models/hv/data/pack_id_scan_log.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2151,6 +2151,36 @@
         </is>
       </c>
     </row>
+    <row r="57" ht="18" customHeight="1">
+      <c r="A57" s="4" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>3:26:18 PM</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>ABA51202605281A00111</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281A00111</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added mongodb atlas updates
</commit_message>
<xml_diff>
--- a/models/hv/data/pack_id_scan_log.xlsx
+++ b/models/hv/data/pack_id_scan_log.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2181,6 +2181,66 @@
         </is>
       </c>
     </row>
+    <row r="58" ht="18" customHeight="1">
+      <c r="A58" s="6" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>11:10:11 AM</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>ABA51202605281A00111</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F58" s="7" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281A00111</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="18" customHeight="1">
+      <c r="A59" s="4" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>11:52:58 AM</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>ABA51202605281A00112</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F59" s="5" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281A00112</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
unwanted code removed from zpl.py and labels.py and the state values changed for set_entry_enabled.
</commit_message>
<xml_diff>
--- a/models/hv/data/pack_id_scan_log.xlsx
+++ b/models/hv/data/pack_id_scan_log.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F68"/>
+  <dimension ref="A1:F69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2511,6 +2511,36 @@
         </is>
       </c>
     </row>
+    <row r="69" ht="18" customHeight="1">
+      <c r="A69" s="4" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>3:58:11 PM</t>
+        </is>
+      </c>
+      <c r="D69" s="5" t="inlineStr">
+        <is>
+          <t>ABA51202605281U00111</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F69" s="5" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U00111</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
scan_log.db created where old scan_log.xlsx kept as it is
</commit_message>
<xml_diff>
--- a/models/hv/data/pack_id_scan_log.xlsx
+++ b/models/hv/data/pack_id_scan_log.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F69"/>
+  <dimension ref="A1:F82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2541,6 +2541,396 @@
         </is>
       </c>
     </row>
+    <row r="70" ht="18" customHeight="1">
+      <c r="A70" s="6" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="inlineStr">
+        <is>
+          <t>4:30:39 PM</t>
+        </is>
+      </c>
+      <c r="D70" s="7" t="inlineStr">
+        <is>
+          <t>ABA51202605281U12345</t>
+        </is>
+      </c>
+      <c r="E70" s="6" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F70" s="7" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U12345</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="18" customHeight="1">
+      <c r="A71" s="4" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>4:32:42 PM</t>
+        </is>
+      </c>
+      <c r="D71" s="5" t="inlineStr">
+        <is>
+          <t>ABA51202605281U12345</t>
+        </is>
+      </c>
+      <c r="E71" s="4" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F71" s="5" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U12345</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="18" customHeight="1">
+      <c r="A72" s="6" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="inlineStr">
+        <is>
+          <t>4:32:58 PM</t>
+        </is>
+      </c>
+      <c r="D72" s="7" t="inlineStr">
+        <is>
+          <t>ABA51202605281U12345</t>
+        </is>
+      </c>
+      <c r="E72" s="6" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F72" s="7" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U12345</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="18" customHeight="1">
+      <c r="A73" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>4:33:15 PM</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>ABA51202605281U12345</t>
+        </is>
+      </c>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F73" s="5" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U12345</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="18" customHeight="1">
+      <c r="A74" s="6" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="inlineStr">
+        <is>
+          <t>4:33:17 PM</t>
+        </is>
+      </c>
+      <c r="D74" s="7" t="inlineStr">
+        <is>
+          <t>ABA51202605281U12345</t>
+        </is>
+      </c>
+      <c r="E74" s="6" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F74" s="7" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U12345</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="18" customHeight="1">
+      <c r="A75" s="4" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>4:33:19 PM</t>
+        </is>
+      </c>
+      <c r="D75" s="5" t="inlineStr">
+        <is>
+          <t>ABA51202605281U12345</t>
+        </is>
+      </c>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F75" s="5" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U12345</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="18" customHeight="1">
+      <c r="A76" s="6" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="inlineStr">
+        <is>
+          <t>4:33:21 PM</t>
+        </is>
+      </c>
+      <c r="D76" s="7" t="inlineStr">
+        <is>
+          <t>ABA51202605281U12345</t>
+        </is>
+      </c>
+      <c r="E76" s="6" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F76" s="7" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U12345</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="18" customHeight="1">
+      <c r="A77" s="4" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>4:33:22 PM</t>
+        </is>
+      </c>
+      <c r="D77" s="5" t="inlineStr">
+        <is>
+          <t>ABA51202605281U12345</t>
+        </is>
+      </c>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F77" s="5" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U12345</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="18" customHeight="1">
+      <c r="A78" s="6" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" s="6" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C78" s="6" t="inlineStr">
+        <is>
+          <t>4:33:26 PM</t>
+        </is>
+      </c>
+      <c r="D78" s="7" t="inlineStr">
+        <is>
+          <t>ABA51202605281U12345</t>
+        </is>
+      </c>
+      <c r="E78" s="6" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F78" s="7" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U12345</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="18" customHeight="1">
+      <c r="A79" s="4" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>4:33:28 PM</t>
+        </is>
+      </c>
+      <c r="D79" s="5" t="inlineStr">
+        <is>
+          <t>ABA51202605281U12345</t>
+        </is>
+      </c>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F79" s="5" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U12345</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="18" customHeight="1">
+      <c r="A80" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" s="6" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C80" s="6" t="inlineStr">
+        <is>
+          <t>4:33:40 PM</t>
+        </is>
+      </c>
+      <c r="D80" s="7" t="inlineStr">
+        <is>
+          <t>ABA51202605281U12345</t>
+        </is>
+      </c>
+      <c r="E80" s="6" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F80" s="7" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U12345</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="18" customHeight="1">
+      <c r="A81" s="4" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>4:33:52 PM</t>
+        </is>
+      </c>
+      <c r="D81" s="5" t="inlineStr">
+        <is>
+          <t>ABA51202605281U12345</t>
+        </is>
+      </c>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F81" s="5" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U12345</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="18" customHeight="1">
+      <c r="A82" s="6" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="inlineStr">
+        <is>
+          <t>4:33:57 PM</t>
+        </is>
+      </c>
+      <c r="D82" s="7" t="inlineStr">
+        <is>
+          <t>ABA51202605281U12345</t>
+        </is>
+      </c>
+      <c r="E82" s="6" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F82" s="7" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U12345</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
some changes before server client updates
</commit_message>
<xml_diff>
--- a/models/hv/data/pack_id_scan_log.xlsx
+++ b/models/hv/data/pack_id_scan_log.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3036" yWindow="2340" windowWidth="11268" windowHeight="9900" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pack ID" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Pack ID" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F71"/>
+  <dimension ref="A1:F75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2601,6 +2601,126 @@
         </is>
       </c>
     </row>
+    <row r="72" ht="18" customHeight="1">
+      <c r="A72" s="6" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="inlineStr">
+        <is>
+          <t>4:40:49 PM</t>
+        </is>
+      </c>
+      <c r="D72" s="7" t="inlineStr">
+        <is>
+          <t>ABA51202605281U00111</t>
+        </is>
+      </c>
+      <c r="E72" s="6" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F72" s="7" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U00111</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="18" customHeight="1">
+      <c r="A73" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>4:58:42 PM</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>ABA51202605281U00111</t>
+        </is>
+      </c>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F73" s="5" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U00111</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="18" customHeight="1">
+      <c r="A74" s="6" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="inlineStr">
+        <is>
+          <t>8:35:47 AM</t>
+        </is>
+      </c>
+      <c r="D74" s="7" t="inlineStr">
+        <is>
+          <t>ABA51202605281U00111</t>
+        </is>
+      </c>
+      <c r="E74" s="6" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F74" s="7" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U00111</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="18" customHeight="1">
+      <c r="A75" s="4" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>11:29:15 AM</t>
+        </is>
+      </c>
+      <c r="D75" s="5" t="inlineStr">
+        <is>
+          <t>ABA51202605281U00111</t>
+        </is>
+      </c>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F75" s="5" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U00111</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
client server files updated, __future__ line removed
</commit_message>
<xml_diff>
--- a/models/hv/data/pack_id_scan_log.xlsx
+++ b/models/hv/data/pack_id_scan_log.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F75"/>
+  <dimension ref="A1:F77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2721,6 +2721,66 @@
         </is>
       </c>
     </row>
+    <row r="76" ht="18" customHeight="1">
+      <c r="A76" s="6" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="inlineStr">
+        <is>
+          <t>2:33:05 PM</t>
+        </is>
+      </c>
+      <c r="D76" s="7" t="inlineStr">
+        <is>
+          <t>ABA51202605281U00111</t>
+        </is>
+      </c>
+      <c r="E76" s="6" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F76" s="7" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U00111</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="18" customHeight="1">
+      <c r="A77" s="4" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>2:33:16 PM</t>
+        </is>
+      </c>
+      <c r="D77" s="5" t="inlineStr">
+        <is>
+          <t>ABA51202605281U00112</t>
+        </is>
+      </c>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F77" s="5" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U00112</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
added api urls option in admin settings and calling api url from that screen
</commit_message>
<xml_diff>
--- a/models/hv/data/pack_id_scan_log.xlsx
+++ b/models/hv/data/pack_id_scan_log.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3036" yWindow="2340" windowWidth="11268" windowHeight="9900" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Pack ID" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pack ID" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F91"/>
+  <dimension ref="A1:F99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3201,6 +3201,246 @@
         </is>
       </c>
     </row>
+    <row r="92" ht="18" customHeight="1">
+      <c r="A92" s="6" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="6" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C92" s="6" t="inlineStr">
+        <is>
+          <t>09:53:56 AM</t>
+        </is>
+      </c>
+      <c r="D92" s="7" t="inlineStr">
+        <is>
+          <t>ABA51202605281U00108</t>
+        </is>
+      </c>
+      <c r="E92" s="6" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F92" s="7" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U00108</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="18" customHeight="1">
+      <c r="A93" s="4" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="4" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C93" s="4" t="inlineStr">
+        <is>
+          <t>09:53:59 AM</t>
+        </is>
+      </c>
+      <c r="D93" s="5" t="inlineStr">
+        <is>
+          <t>ABA51202605281U00105</t>
+        </is>
+      </c>
+      <c r="E93" s="4" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F93" s="5" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U00105</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="18" customHeight="1">
+      <c r="A94" s="6" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" s="6" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C94" s="6" t="inlineStr">
+        <is>
+          <t>09:54:02 AM</t>
+        </is>
+      </c>
+      <c r="D94" s="7" t="inlineStr">
+        <is>
+          <t>ABA51202605281U00109</t>
+        </is>
+      </c>
+      <c r="E94" s="6" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F94" s="7" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U00109</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="18" customHeight="1">
+      <c r="A95" s="4" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" s="4" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C95" s="4" t="inlineStr">
+        <is>
+          <t>09:54:09 AM</t>
+        </is>
+      </c>
+      <c r="D95" s="5" t="inlineStr">
+        <is>
+          <t>ABA51202605281U00101</t>
+        </is>
+      </c>
+      <c r="E95" s="4" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F95" s="5" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U00101</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="18" customHeight="1">
+      <c r="A96" s="6" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" s="6" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C96" s="6" t="inlineStr">
+        <is>
+          <t>09:55:51 AM</t>
+        </is>
+      </c>
+      <c r="D96" s="7" t="inlineStr">
+        <is>
+          <t>ABA51202605281U00108</t>
+        </is>
+      </c>
+      <c r="E96" s="6" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F96" s="7" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U00108</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="18" customHeight="1">
+      <c r="A97" s="4" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" s="4" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C97" s="4" t="inlineStr">
+        <is>
+          <t>09:56:51 AM</t>
+        </is>
+      </c>
+      <c r="D97" s="5" t="inlineStr">
+        <is>
+          <t>ABA51202605281U00100</t>
+        </is>
+      </c>
+      <c r="E97" s="4" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F97" s="5" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U00100</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="18" customHeight="1">
+      <c r="A98" s="6" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" s="6" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C98" s="6" t="inlineStr">
+        <is>
+          <t>11:23:59 AM</t>
+        </is>
+      </c>
+      <c r="D98" s="7" t="inlineStr">
+        <is>
+          <t>ABA51202605281U00108</t>
+        </is>
+      </c>
+      <c r="E98" s="6" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F98" s="7" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U00108</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="18" customHeight="1">
+      <c r="A99" s="4" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" s="4" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C99" s="4" t="inlineStr">
+        <is>
+          <t>11:53:23 AM</t>
+        </is>
+      </c>
+      <c r="D99" s="5" t="inlineStr">
+        <is>
+          <t>ABA51202605281U00101</t>
+        </is>
+      </c>
+      <c r="E99" s="4" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F99" s="5" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U00101</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
resequence logic for sl.no updated
</commit_message>
<xml_diff>
--- a/models/hv/data/pack_id_scan_log.xlsx
+++ b/models/hv/data/pack_id_scan_log.xlsx
@@ -458,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F115"/>
+  <dimension ref="A1:F117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3921,6 +3921,66 @@
         </is>
       </c>
     </row>
+    <row r="116" ht="18" customHeight="1">
+      <c r="A116" s="6" t="n">
+        <v>115</v>
+      </c>
+      <c r="B116" s="6" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C116" s="6" t="inlineStr">
+        <is>
+          <t>11:39:20 AM</t>
+        </is>
+      </c>
+      <c r="D116" s="7" t="inlineStr">
+        <is>
+          <t>ABA51202605281U00134</t>
+        </is>
+      </c>
+      <c r="E116" s="6" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F116" s="7" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U00134</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="18" customHeight="1">
+      <c r="A117" s="4" t="n">
+        <v>116</v>
+      </c>
+      <c r="B117" s="4" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C117" s="4" t="inlineStr">
+        <is>
+          <t>11:41:14 AM</t>
+        </is>
+      </c>
+      <c r="D117" s="5" t="inlineStr">
+        <is>
+          <t>ABA51202605281U00134</t>
+        </is>
+      </c>
+      <c r="E117" s="4" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F117" s="5" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U00134</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
machine name and machine id variables added to excel columns at the end and get the value from admi settings notebook in api settings frame.
</commit_message>
<xml_diff>
--- a/models/hv/data/pack_id_scan_log.xlsx
+++ b/models/hv/data/pack_id_scan_log.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,8 +34,14 @@
       <name val="Segoe UI"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -57,6 +63,11 @@
         <fgColor rgb="00EEF2F7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -70,7 +81,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -92,6 +103,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -458,8 +472,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F117"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <dimension ref="A1:H119"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelCol="0"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -467,9 +481,11 @@
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28.05" customHeight="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Sl.No</t>
@@ -498,6 +514,16 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Pack QR Data</t>
+        </is>
+      </c>
+      <c r="G1" s="8" t="inlineStr">
+        <is>
+          <t>Machine Name</t>
+        </is>
+      </c>
+      <c r="H1" s="8" t="inlineStr">
+        <is>
+          <t>Machine ID</t>
         </is>
       </c>
     </row>
@@ -3978,6 +4004,86 @@
       <c r="F117" s="5" t="inlineStr">
         <is>
           <t>VX156060:ABA51202605281U00134</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="18" customHeight="1">
+      <c r="A118" s="6" t="n">
+        <v>117</v>
+      </c>
+      <c r="B118" s="6" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C118" s="6" t="inlineStr">
+        <is>
+          <t>12:44:10 PM</t>
+        </is>
+      </c>
+      <c r="D118" s="7" t="inlineStr">
+        <is>
+          <t>ABA51202605281U00134</t>
+        </is>
+      </c>
+      <c r="E118" s="6" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F118" s="7" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U00134</t>
+        </is>
+      </c>
+      <c r="G118" s="6" t="inlineStr">
+        <is>
+          <t>bat_pc</t>
+        </is>
+      </c>
+      <c r="H118" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="18" customHeight="1">
+      <c r="A119" s="4" t="n">
+        <v>118</v>
+      </c>
+      <c r="B119" s="4" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C119" s="4" t="inlineStr">
+        <is>
+          <t>12:45:53 PM</t>
+        </is>
+      </c>
+      <c r="D119" s="5" t="inlineStr">
+        <is>
+          <t>ABA51202605281U00134</t>
+        </is>
+      </c>
+      <c r="E119" s="4" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F119" s="5" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U00134</t>
+        </is>
+      </c>
+      <c r="G119" s="4" t="inlineStr">
+        <is>
+          <t>bat_pc</t>
+        </is>
+      </c>
+      <c r="H119" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
code optimization- unnecessary code removed and commented lines removed
</commit_message>
<xml_diff>
--- a/models/hv/data/pack_id_scan_log.xlsx
+++ b/models/hv/data/pack_id_scan_log.xlsx
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H150"/>
+  <dimension ref="A1:H154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelCol="0"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5199,6 +5199,142 @@
       <c r="G150" s="6" t="inlineStr"/>
       <c r="H150" s="6" t="inlineStr"/>
     </row>
+    <row r="151" ht="18" customHeight="1">
+      <c r="A151" s="4" t="n">
+        <v>150</v>
+      </c>
+      <c r="B151" s="4" t="inlineStr">
+        <is>
+          <t>25 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C151" s="4" t="inlineStr">
+        <is>
+          <t>10:31:47 AM</t>
+        </is>
+      </c>
+      <c r="D151" s="5" t="inlineStr">
+        <is>
+          <t>ABA41202609251R00297</t>
+        </is>
+      </c>
+      <c r="E151" s="4" t="inlineStr">
+        <is>
+          <t>16P</t>
+        </is>
+      </c>
+      <c r="F151" s="5" t="inlineStr">
+        <is>
+          <t>VQ150010:ABA41202609251R00297</t>
+        </is>
+      </c>
+      <c r="G151" s="4" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="H151" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="152" ht="18" customHeight="1">
+      <c r="A152" s="6" t="n">
+        <v>151</v>
+      </c>
+      <c r="B152" s="6" t="inlineStr">
+        <is>
+          <t>15 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C152" s="6" t="inlineStr">
+        <is>
+          <t>10:52:03 AM</t>
+        </is>
+      </c>
+      <c r="D152" s="7" t="inlineStr">
+        <is>
+          <t>ABA61202609151R00276</t>
+        </is>
+      </c>
+      <c r="E152" s="6" t="inlineStr">
+        <is>
+          <t>27P</t>
+        </is>
+      </c>
+      <c r="F152" s="7" t="inlineStr">
+        <is>
+          <t>VQ150030:ABA61202609151R00276</t>
+        </is>
+      </c>
+      <c r="G152" s="6" t="inlineStr"/>
+      <c r="H152" s="6" t="inlineStr"/>
+    </row>
+    <row r="153" ht="18" customHeight="1">
+      <c r="A153" s="4" t="n">
+        <v>152</v>
+      </c>
+      <c r="B153" s="4" t="inlineStr">
+        <is>
+          <t>15 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C153" s="4" t="inlineStr">
+        <is>
+          <t>02:33:31 PM</t>
+        </is>
+      </c>
+      <c r="D153" s="5" t="inlineStr">
+        <is>
+          <t>ABA61202609151R00276</t>
+        </is>
+      </c>
+      <c r="E153" s="4" t="inlineStr">
+        <is>
+          <t>27P</t>
+        </is>
+      </c>
+      <c r="F153" s="5" t="inlineStr">
+        <is>
+          <t>VQ150030:ABA61202609151R00276</t>
+        </is>
+      </c>
+      <c r="G153" s="4" t="inlineStr"/>
+      <c r="H153" s="4" t="inlineStr"/>
+    </row>
+    <row r="154" ht="18" customHeight="1">
+      <c r="A154" s="6" t="n">
+        <v>153</v>
+      </c>
+      <c r="B154" s="6" t="inlineStr">
+        <is>
+          <t>15 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C154" s="6" t="inlineStr">
+        <is>
+          <t>02:34:12 PM</t>
+        </is>
+      </c>
+      <c r="D154" s="7" t="inlineStr">
+        <is>
+          <t>ABA61202609151R00276</t>
+        </is>
+      </c>
+      <c r="E154" s="6" t="inlineStr">
+        <is>
+          <t>27P</t>
+        </is>
+      </c>
+      <c r="F154" s="7" t="inlineStr">
+        <is>
+          <t>VQ150030:ABA61202609151R00276</t>
+        </is>
+      </c>
+      <c r="G154" s="6" t="inlineStr"/>
+      <c r="H154" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
zpl code for domestic and export will be updated based on category and tac will be removed for export category in build_battery_pack_id_zpl_unified
</commit_message>
<xml_diff>
--- a/models/hv/data/pack_id_scan_log.xlsx
+++ b/models/hv/data/pack_id_scan_log.xlsx
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H154"/>
+  <dimension ref="A1:H160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelCol="0"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5335,6 +5335,198 @@
       <c r="G154" s="6" t="inlineStr"/>
       <c r="H154" s="6" t="inlineStr"/>
     </row>
+    <row r="155" ht="18" customHeight="1">
+      <c r="A155" s="4" t="n">
+        <v>154</v>
+      </c>
+      <c r="B155" s="4" t="inlineStr">
+        <is>
+          <t>24 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C155" s="4" t="inlineStr">
+        <is>
+          <t>04:19:00 PM</t>
+        </is>
+      </c>
+      <c r="D155" s="5" t="inlineStr">
+        <is>
+          <t>ABA31202609241R00295</t>
+        </is>
+      </c>
+      <c r="E155" s="4" t="inlineStr">
+        <is>
+          <t>12P</t>
+        </is>
+      </c>
+      <c r="F155" s="5" t="inlineStr">
+        <is>
+          <t>VQ150000:ABA31202609241R00295</t>
+        </is>
+      </c>
+      <c r="G155" s="4" t="inlineStr"/>
+      <c r="H155" s="4" t="inlineStr"/>
+    </row>
+    <row r="156" ht="18" customHeight="1">
+      <c r="A156" s="6" t="n">
+        <v>155</v>
+      </c>
+      <c r="B156" s="6" t="inlineStr">
+        <is>
+          <t>24 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C156" s="6" t="inlineStr">
+        <is>
+          <t>04:33:10 PM</t>
+        </is>
+      </c>
+      <c r="D156" s="7" t="inlineStr">
+        <is>
+          <t>ABA31202609242R00295</t>
+        </is>
+      </c>
+      <c r="E156" s="6" t="inlineStr">
+        <is>
+          <t>12P</t>
+        </is>
+      </c>
+      <c r="F156" s="7" t="inlineStr">
+        <is>
+          <t>VQ150000:ABA31202609242R00295</t>
+        </is>
+      </c>
+      <c r="G156" s="6" t="inlineStr"/>
+      <c r="H156" s="6" t="inlineStr"/>
+    </row>
+    <row r="157" ht="18" customHeight="1">
+      <c r="A157" s="4" t="n">
+        <v>156</v>
+      </c>
+      <c r="B157" s="4" t="inlineStr">
+        <is>
+          <t>24 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C157" s="4" t="inlineStr">
+        <is>
+          <t>04:33:18 PM</t>
+        </is>
+      </c>
+      <c r="D157" s="5" t="inlineStr">
+        <is>
+          <t>ABA31202609242R00295</t>
+        </is>
+      </c>
+      <c r="E157" s="4" t="inlineStr">
+        <is>
+          <t>12P</t>
+        </is>
+      </c>
+      <c r="F157" s="5" t="inlineStr">
+        <is>
+          <t>VQ150000:ABA31202609242R00295</t>
+        </is>
+      </c>
+      <c r="G157" s="4" t="inlineStr"/>
+      <c r="H157" s="4" t="inlineStr"/>
+    </row>
+    <row r="158" ht="18" customHeight="1">
+      <c r="A158" s="6" t="n">
+        <v>157</v>
+      </c>
+      <c r="B158" s="6" t="inlineStr">
+        <is>
+          <t>24 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C158" s="6" t="inlineStr">
+        <is>
+          <t>04:36:20 PM</t>
+        </is>
+      </c>
+      <c r="D158" s="7" t="inlineStr">
+        <is>
+          <t>ABA31202609242R00295</t>
+        </is>
+      </c>
+      <c r="E158" s="6" t="inlineStr">
+        <is>
+          <t>12P</t>
+        </is>
+      </c>
+      <c r="F158" s="7" t="inlineStr">
+        <is>
+          <t>VQ150000:ABA31202609242R00295</t>
+        </is>
+      </c>
+      <c r="G158" s="6" t="inlineStr"/>
+      <c r="H158" s="6" t="inlineStr"/>
+    </row>
+    <row r="159" ht="18" customHeight="1">
+      <c r="A159" s="4" t="n">
+        <v>158</v>
+      </c>
+      <c r="B159" s="4" t="inlineStr">
+        <is>
+          <t>24 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C159" s="4" t="inlineStr">
+        <is>
+          <t>04:45:32 PM</t>
+        </is>
+      </c>
+      <c r="D159" s="5" t="inlineStr">
+        <is>
+          <t>ABA31202609242R00295</t>
+        </is>
+      </c>
+      <c r="E159" s="4" t="inlineStr">
+        <is>
+          <t>12P</t>
+        </is>
+      </c>
+      <c r="F159" s="5" t="inlineStr">
+        <is>
+          <t>VQ150000:ABA31202609242R00295</t>
+        </is>
+      </c>
+      <c r="G159" s="4" t="inlineStr"/>
+      <c r="H159" s="4" t="inlineStr"/>
+    </row>
+    <row r="160" ht="18" customHeight="1">
+      <c r="A160" s="6" t="n">
+        <v>159</v>
+      </c>
+      <c r="B160" s="6" t="inlineStr">
+        <is>
+          <t>24 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C160" s="6" t="inlineStr">
+        <is>
+          <t>04:53:05 PM</t>
+        </is>
+      </c>
+      <c r="D160" s="7" t="inlineStr">
+        <is>
+          <t>ABA31202609242R00295</t>
+        </is>
+      </c>
+      <c r="E160" s="6" t="inlineStr">
+        <is>
+          <t>12P</t>
+        </is>
+      </c>
+      <c r="F160" s="7" t="inlineStr">
+        <is>
+          <t>VQ150000:ABA31202609242R00295</t>
+        </is>
+      </c>
+      <c r="G160" s="6" t="inlineStr"/>
+      <c r="H160" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
col_idx mentioned in _build_header in pack_id_scan_log.py to enamurate the sl for every newly added rows
</commit_message>
<xml_diff>
--- a/models/hv/data/pack_id_scan_log.xlsx
+++ b/models/hv/data/pack_id_scan_log.xlsx
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H160"/>
+  <dimension ref="A1:H171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelCol="0"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5527,6 +5527,390 @@
       <c r="G160" s="6" t="inlineStr"/>
       <c r="H160" s="6" t="inlineStr"/>
     </row>
+    <row r="161" ht="18" customHeight="1">
+      <c r="A161" s="4" t="n">
+        <v>160</v>
+      </c>
+      <c r="B161" s="4" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C161" s="4" t="inlineStr">
+        <is>
+          <t>09:33:42 AM</t>
+        </is>
+      </c>
+      <c r="D161" s="5" t="inlineStr">
+        <is>
+          <t>ABA51202605281U00134</t>
+        </is>
+      </c>
+      <c r="E161" s="4" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F161" s="5" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U00134</t>
+        </is>
+      </c>
+      <c r="G161" s="4" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="H161" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="162" ht="18" customHeight="1">
+      <c r="A162" s="6" t="n">
+        <v>161</v>
+      </c>
+      <c r="B162" s="6" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C162" s="6" t="inlineStr">
+        <is>
+          <t>09:36:03 AM</t>
+        </is>
+      </c>
+      <c r="D162" s="7" t="inlineStr">
+        <is>
+          <t>ABA51202605281U00137</t>
+        </is>
+      </c>
+      <c r="E162" s="6" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F162" s="7" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U00137</t>
+        </is>
+      </c>
+      <c r="G162" s="6" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="H162" s="6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" ht="18" customHeight="1">
+      <c r="A163" s="4" t="n">
+        <v>162</v>
+      </c>
+      <c r="B163" s="4" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C163" s="4" t="inlineStr">
+        <is>
+          <t>09:55:24 AM</t>
+        </is>
+      </c>
+      <c r="D163" s="5" t="inlineStr">
+        <is>
+          <t>ABA51202605281U00137</t>
+        </is>
+      </c>
+      <c r="E163" s="4" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F163" s="5" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U00137</t>
+        </is>
+      </c>
+      <c r="G163" s="4" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="H163" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="164" ht="18" customHeight="1">
+      <c r="A164" s="6" t="n">
+        <v>163</v>
+      </c>
+      <c r="B164" s="6" t="inlineStr">
+        <is>
+          <t>28 May 2026</t>
+        </is>
+      </c>
+      <c r="C164" s="6" t="inlineStr">
+        <is>
+          <t>09:59:07 AM</t>
+        </is>
+      </c>
+      <c r="D164" s="7" t="inlineStr">
+        <is>
+          <t>ABA51202605281U00137</t>
+        </is>
+      </c>
+      <c r="E164" s="6" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F164" s="7" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202605281U00137</t>
+        </is>
+      </c>
+      <c r="G164" s="6" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="H164" s="6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="165" ht="18" customHeight="1">
+      <c r="A165" s="4" t="n">
+        <v>164</v>
+      </c>
+      <c r="B165" s="4" t="inlineStr">
+        <is>
+          <t>15 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C165" s="4" t="inlineStr">
+        <is>
+          <t>11:15:41 AM</t>
+        </is>
+      </c>
+      <c r="D165" s="5" t="inlineStr">
+        <is>
+          <t>ABA61202609151R00276</t>
+        </is>
+      </c>
+      <c r="E165" s="4" t="inlineStr">
+        <is>
+          <t>27P</t>
+        </is>
+      </c>
+      <c r="F165" s="5" t="inlineStr">
+        <is>
+          <t>VQ150030:ABA61202609151R00276</t>
+        </is>
+      </c>
+      <c r="G165" s="4" t="inlineStr"/>
+      <c r="H165" s="4" t="inlineStr"/>
+    </row>
+    <row r="166" ht="18" customHeight="1">
+      <c r="A166" s="6" t="n">
+        <v>165</v>
+      </c>
+      <c r="B166" s="6" t="inlineStr">
+        <is>
+          <t>24 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C166" s="6" t="inlineStr">
+        <is>
+          <t>11:26:04 AM</t>
+        </is>
+      </c>
+      <c r="D166" s="7" t="inlineStr">
+        <is>
+          <t>ABA31202609241R00295</t>
+        </is>
+      </c>
+      <c r="E166" s="6" t="inlineStr">
+        <is>
+          <t>12P</t>
+        </is>
+      </c>
+      <c r="F166" s="7" t="inlineStr">
+        <is>
+          <t>VQ150000:ABA31202609241R00295</t>
+        </is>
+      </c>
+      <c r="G166" s="6" t="inlineStr"/>
+      <c r="H166" s="6" t="inlineStr"/>
+    </row>
+    <row r="167" ht="18" customHeight="1">
+      <c r="A167" s="4" t="n">
+        <v>166</v>
+      </c>
+      <c r="B167" s="4" t="inlineStr">
+        <is>
+          <t>25 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C167" s="4" t="inlineStr">
+        <is>
+          <t>11:26:24 AM</t>
+        </is>
+      </c>
+      <c r="D167" s="5" t="inlineStr">
+        <is>
+          <t>ABA41202609251R00297</t>
+        </is>
+      </c>
+      <c r="E167" s="4" t="inlineStr">
+        <is>
+          <t>16P</t>
+        </is>
+      </c>
+      <c r="F167" s="5" t="inlineStr">
+        <is>
+          <t>VQ150010:ABA41202609251R00297</t>
+        </is>
+      </c>
+      <c r="G167" s="4" t="inlineStr"/>
+      <c r="H167" s="4" t="inlineStr"/>
+    </row>
+    <row r="168" ht="18" customHeight="1">
+      <c r="A168" s="6" t="n">
+        <v>167</v>
+      </c>
+      <c r="B168" s="6" t="inlineStr">
+        <is>
+          <t>26 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C168" s="6" t="inlineStr">
+        <is>
+          <t>11:26:35 AM</t>
+        </is>
+      </c>
+      <c r="D168" s="7" t="inlineStr">
+        <is>
+          <t>ABA51202609261R00299</t>
+        </is>
+      </c>
+      <c r="E168" s="6" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F168" s="7" t="inlineStr">
+        <is>
+          <t>VQ150020:ABA51202609261R00299</t>
+        </is>
+      </c>
+      <c r="G168" s="6" t="inlineStr"/>
+      <c r="H168" s="6" t="inlineStr"/>
+    </row>
+    <row r="169" ht="18" customHeight="1">
+      <c r="A169" s="4" t="n">
+        <v>168</v>
+      </c>
+      <c r="B169" s="4" t="inlineStr">
+        <is>
+          <t>15 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C169" s="4" t="inlineStr">
+        <is>
+          <t>11:26:45 AM</t>
+        </is>
+      </c>
+      <c r="D169" s="5" t="inlineStr">
+        <is>
+          <t>ABA61202609151R00277</t>
+        </is>
+      </c>
+      <c r="E169" s="4" t="inlineStr">
+        <is>
+          <t>27P</t>
+        </is>
+      </c>
+      <c r="F169" s="5" t="inlineStr">
+        <is>
+          <t>VQ150030:ABA61202609151R00277</t>
+        </is>
+      </c>
+      <c r="G169" s="4" t="inlineStr"/>
+      <c r="H169" s="4" t="inlineStr"/>
+    </row>
+    <row r="170" ht="18" customHeight="1">
+      <c r="A170" s="6" t="n">
+        <v>169</v>
+      </c>
+      <c r="B170" s="6" t="inlineStr">
+        <is>
+          <t>12 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C170" s="6" t="inlineStr">
+        <is>
+          <t>11:26:53 AM</t>
+        </is>
+      </c>
+      <c r="D170" s="7" t="inlineStr">
+        <is>
+          <t>ABA61202610121R00330</t>
+        </is>
+      </c>
+      <c r="E170" s="6" t="inlineStr">
+        <is>
+          <t>27P</t>
+        </is>
+      </c>
+      <c r="F170" s="7" t="inlineStr">
+        <is>
+          <t>VQ150030:ABA61202610121R00330</t>
+        </is>
+      </c>
+      <c r="G170" s="6" t="inlineStr"/>
+      <c r="H170" s="6" t="inlineStr"/>
+    </row>
+    <row r="171" ht="18" customHeight="1">
+      <c r="A171" s="4" t="n">
+        <v>170</v>
+      </c>
+      <c r="B171" s="4" t="inlineStr">
+        <is>
+          <t>15 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C171" s="4" t="inlineStr">
+        <is>
+          <t>11:27:04 AM</t>
+        </is>
+      </c>
+      <c r="D171" s="5" t="inlineStr">
+        <is>
+          <t>ABA61202609151R00276</t>
+        </is>
+      </c>
+      <c r="E171" s="4" t="inlineStr">
+        <is>
+          <t>27P</t>
+        </is>
+      </c>
+      <c r="F171" s="5" t="inlineStr">
+        <is>
+          <t>VQ150030:ABA61202609151R00276</t>
+        </is>
+      </c>
+      <c r="G171" s="4" t="inlineStr"/>
+      <c r="H171" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
scanner.py changed to make suitable for barcode + enter type scanners
</commit_message>
<xml_diff>
--- a/models/hv/data/pack_id_scan_log.xlsx
+++ b/models/hv/data/pack_id_scan_log.xlsx
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H226"/>
+  <dimension ref="A1:H230"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelCol="0"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -7671,6 +7671,134 @@
       <c r="G226" s="6" t="inlineStr"/>
       <c r="H226" s="6" t="inlineStr"/>
     </row>
+    <row r="227" ht="18" customHeight="1">
+      <c r="A227" s="4" t="n">
+        <v>226</v>
+      </c>
+      <c r="B227" s="4" t="inlineStr">
+        <is>
+          <t>16 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C227" s="4" t="inlineStr">
+        <is>
+          <t>03:25:50 PM</t>
+        </is>
+      </c>
+      <c r="D227" s="5" t="inlineStr">
+        <is>
+          <t>ABA51202609162S00279</t>
+        </is>
+      </c>
+      <c r="E227" s="4" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F227" s="5" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202609162S00279</t>
+        </is>
+      </c>
+      <c r="G227" s="4" t="inlineStr"/>
+      <c r="H227" s="4" t="inlineStr"/>
+    </row>
+    <row r="228" ht="18" customHeight="1">
+      <c r="A228" s="6" t="n">
+        <v>227</v>
+      </c>
+      <c r="B228" s="6" t="inlineStr">
+        <is>
+          <t>16 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C228" s="6" t="inlineStr">
+        <is>
+          <t>03:26:49 PM</t>
+        </is>
+      </c>
+      <c r="D228" s="7" t="inlineStr">
+        <is>
+          <t>ABA51202609162S00279</t>
+        </is>
+      </c>
+      <c r="E228" s="6" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F228" s="7" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202609162S00279</t>
+        </is>
+      </c>
+      <c r="G228" s="6" t="inlineStr"/>
+      <c r="H228" s="6" t="inlineStr"/>
+    </row>
+    <row r="229" ht="18" customHeight="1">
+      <c r="A229" s="4" t="n">
+        <v>228</v>
+      </c>
+      <c r="B229" s="4" t="inlineStr">
+        <is>
+          <t>16 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C229" s="4" t="inlineStr">
+        <is>
+          <t>03:27:48 PM</t>
+        </is>
+      </c>
+      <c r="D229" s="5" t="inlineStr">
+        <is>
+          <t>ABA51202609162S00279</t>
+        </is>
+      </c>
+      <c r="E229" s="4" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F229" s="5" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202609162S00279</t>
+        </is>
+      </c>
+      <c r="G229" s="4" t="inlineStr"/>
+      <c r="H229" s="4" t="inlineStr"/>
+    </row>
+    <row r="230" ht="18" customHeight="1">
+      <c r="A230" s="6" t="n">
+        <v>229</v>
+      </c>
+      <c r="B230" s="6" t="inlineStr">
+        <is>
+          <t>16 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C230" s="6" t="inlineStr">
+        <is>
+          <t>03:28:33 PM</t>
+        </is>
+      </c>
+      <c r="D230" s="7" t="inlineStr">
+        <is>
+          <t>ABA51202609162S00279</t>
+        </is>
+      </c>
+      <c r="E230" s="6" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F230" s="7" t="inlineStr">
+        <is>
+          <t>VQ150020:ABA51202609162S00279</t>
+        </is>
+      </c>
+      <c r="G230" s="6" t="inlineStr"/>
+      <c r="H230" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
test case to add new variant and its other parameters
</commit_message>
<xml_diff>
--- a/models/hv/data/pack_id_scan_log.xlsx
+++ b/models/hv/data/pack_id_scan_log.xlsx
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H230"/>
+  <dimension ref="A1:H233"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelCol="0"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -7799,6 +7799,102 @@
       <c r="G230" s="6" t="inlineStr"/>
       <c r="H230" s="6" t="inlineStr"/>
     </row>
+    <row r="231" ht="18" customHeight="1">
+      <c r="A231" s="4" t="n">
+        <v>230</v>
+      </c>
+      <c r="B231" s="4" t="inlineStr">
+        <is>
+          <t>29 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C231" s="4" t="inlineStr">
+        <is>
+          <t>04:18:22 PM</t>
+        </is>
+      </c>
+      <c r="D231" s="5" t="inlineStr">
+        <is>
+          <t>ABS11202610291U00002</t>
+        </is>
+      </c>
+      <c r="E231" s="4" t="inlineStr">
+        <is>
+          <t>SW_LH_8P</t>
+        </is>
+      </c>
+      <c r="F231" s="5" t="inlineStr">
+        <is>
+          <t>VX155810:ABS11202610291U00002</t>
+        </is>
+      </c>
+      <c r="G231" s="4" t="inlineStr"/>
+      <c r="H231" s="4" t="inlineStr"/>
+    </row>
+    <row r="232" ht="18" customHeight="1">
+      <c r="A232" s="6" t="n">
+        <v>231</v>
+      </c>
+      <c r="B232" s="6" t="inlineStr">
+        <is>
+          <t>29 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C232" s="6" t="inlineStr">
+        <is>
+          <t>04:29:26 PM</t>
+        </is>
+      </c>
+      <c r="D232" s="7" t="inlineStr">
+        <is>
+          <t>ABS11202610291U00002</t>
+        </is>
+      </c>
+      <c r="E232" s="6" t="inlineStr">
+        <is>
+          <t>SW_LH_8P</t>
+        </is>
+      </c>
+      <c r="F232" s="7" t="inlineStr">
+        <is>
+          <t>VX155810:ABS11202610291U00002</t>
+        </is>
+      </c>
+      <c r="G232" s="6" t="inlineStr"/>
+      <c r="H232" s="6" t="inlineStr"/>
+    </row>
+    <row r="233" ht="18" customHeight="1">
+      <c r="A233" s="4" t="n">
+        <v>232</v>
+      </c>
+      <c r="B233" s="4" t="inlineStr">
+        <is>
+          <t>29 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C233" s="4" t="inlineStr">
+        <is>
+          <t>04:30:56 PM</t>
+        </is>
+      </c>
+      <c r="D233" s="5" t="inlineStr">
+        <is>
+          <t>ABS11202610291U00002</t>
+        </is>
+      </c>
+      <c r="E233" s="4" t="inlineStr">
+        <is>
+          <t>SW_LH_8P</t>
+        </is>
+      </c>
+      <c r="F233" s="5" t="inlineStr">
+        <is>
+          <t>VX155810:ABS11202610291U00002</t>
+        </is>
+      </c>
+      <c r="G233" s="4" t="inlineStr"/>
+      <c r="H233" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
new formats added and simplifies code and written steps.txt to add new variants to project
</commit_message>
<xml_diff>
--- a/models/hv/data/pack_id_scan_log.xlsx
+++ b/models/hv/data/pack_id_scan_log.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3036" yWindow="2340" windowWidth="11268" windowHeight="9900" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pack ID" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Pack ID" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H233"/>
+  <dimension ref="A1:H240"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelCol="0"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -7895,6 +7895,230 @@
       <c r="G233" s="4" t="inlineStr"/>
       <c r="H233" s="4" t="inlineStr"/>
     </row>
+    <row r="234" ht="18" customHeight="1">
+      <c r="A234" s="6" t="n">
+        <v>233</v>
+      </c>
+      <c r="B234" s="6" t="inlineStr">
+        <is>
+          <t>29 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C234" s="6" t="inlineStr">
+        <is>
+          <t>09:07:11 PM</t>
+        </is>
+      </c>
+      <c r="D234" s="7" t="inlineStr">
+        <is>
+          <t>ABS11202610291R00108</t>
+        </is>
+      </c>
+      <c r="E234" s="6" t="inlineStr">
+        <is>
+          <t>SW_LH_8P</t>
+        </is>
+      </c>
+      <c r="F234" s="7" t="inlineStr">
+        <is>
+          <t>BP00000129:ABS11202610291R00108</t>
+        </is>
+      </c>
+      <c r="G234" s="6" t="inlineStr"/>
+      <c r="H234" s="6" t="inlineStr"/>
+    </row>
+    <row r="235" ht="18" customHeight="1">
+      <c r="A235" s="4" t="n">
+        <v>234</v>
+      </c>
+      <c r="B235" s="4" t="inlineStr">
+        <is>
+          <t>29 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C235" s="4" t="inlineStr">
+        <is>
+          <t>09:17:24 PM</t>
+        </is>
+      </c>
+      <c r="D235" s="5" t="inlineStr">
+        <is>
+          <t>ACS11202610291R00001</t>
+        </is>
+      </c>
+      <c r="E235" s="4" t="inlineStr">
+        <is>
+          <t>SW_LH_8P</t>
+        </is>
+      </c>
+      <c r="F235" s="5" t="inlineStr">
+        <is>
+          <t>BP00000129:ACS11202610291R00001</t>
+        </is>
+      </c>
+      <c r="G235" s="4" t="inlineStr"/>
+      <c r="H235" s="4" t="inlineStr"/>
+    </row>
+    <row r="236" ht="18" customHeight="1">
+      <c r="A236" s="6" t="n">
+        <v>235</v>
+      </c>
+      <c r="B236" s="6" t="inlineStr">
+        <is>
+          <t>29 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C236" s="6" t="inlineStr">
+        <is>
+          <t>10:05:58 PM</t>
+        </is>
+      </c>
+      <c r="D236" s="7" t="inlineStr">
+        <is>
+          <t>ACS11202610291U00010</t>
+        </is>
+      </c>
+      <c r="E236" s="6" t="inlineStr">
+        <is>
+          <t>SW_LH_8P</t>
+        </is>
+      </c>
+      <c r="F236" s="7" t="inlineStr">
+        <is>
+          <t>BP00000129:ACS11202610291U00010</t>
+        </is>
+      </c>
+      <c r="G236" s="6" t="inlineStr"/>
+      <c r="H236" s="6" t="inlineStr"/>
+    </row>
+    <row r="237" ht="18" customHeight="1">
+      <c r="A237" s="4" t="n">
+        <v>236</v>
+      </c>
+      <c r="B237" s="4" t="inlineStr">
+        <is>
+          <t>29 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C237" s="4" t="inlineStr">
+        <is>
+          <t>10:07:35 PM</t>
+        </is>
+      </c>
+      <c r="D237" s="5" t="inlineStr">
+        <is>
+          <t>ACS11202610292U00010</t>
+        </is>
+      </c>
+      <c r="E237" s="4" t="inlineStr">
+        <is>
+          <t>SW_LH_8P</t>
+        </is>
+      </c>
+      <c r="F237" s="5" t="inlineStr">
+        <is>
+          <t>BP00000129:ACS11202610292U00010</t>
+        </is>
+      </c>
+      <c r="G237" s="4" t="inlineStr"/>
+      <c r="H237" s="4" t="inlineStr"/>
+    </row>
+    <row r="238" ht="18" customHeight="1">
+      <c r="A238" s="6" t="n">
+        <v>237</v>
+      </c>
+      <c r="B238" s="6" t="inlineStr">
+        <is>
+          <t>29 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C238" s="6" t="inlineStr">
+        <is>
+          <t>10:12:44 PM</t>
+        </is>
+      </c>
+      <c r="D238" s="7" t="inlineStr">
+        <is>
+          <t>ACS11202610291U00011</t>
+        </is>
+      </c>
+      <c r="E238" s="6" t="inlineStr">
+        <is>
+          <t>SW_LH_8P</t>
+        </is>
+      </c>
+      <c r="F238" s="7" t="inlineStr">
+        <is>
+          <t>BP00000129:ACS11202610291U00011</t>
+        </is>
+      </c>
+      <c r="G238" s="6" t="inlineStr"/>
+      <c r="H238" s="6" t="inlineStr"/>
+    </row>
+    <row r="239" ht="18" customHeight="1">
+      <c r="A239" s="4" t="n">
+        <v>238</v>
+      </c>
+      <c r="B239" s="4" t="inlineStr">
+        <is>
+          <t>29 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C239" s="4" t="inlineStr">
+        <is>
+          <t>10:15:45 PM</t>
+        </is>
+      </c>
+      <c r="D239" s="5" t="inlineStr">
+        <is>
+          <t>ACS11202610291U00012</t>
+        </is>
+      </c>
+      <c r="E239" s="4" t="inlineStr">
+        <is>
+          <t>SW_LH_8P</t>
+        </is>
+      </c>
+      <c r="F239" s="5" t="inlineStr">
+        <is>
+          <t>BP00000129:ACS11202610291U00012</t>
+        </is>
+      </c>
+      <c r="G239" s="4" t="inlineStr"/>
+      <c r="H239" s="4" t="inlineStr"/>
+    </row>
+    <row r="240" ht="18" customHeight="1">
+      <c r="A240" s="6" t="n">
+        <v>239</v>
+      </c>
+      <c r="B240" s="6" t="inlineStr">
+        <is>
+          <t>29 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C240" s="6" t="inlineStr">
+        <is>
+          <t>10:16:49 PM</t>
+        </is>
+      </c>
+      <c r="D240" s="7" t="inlineStr">
+        <is>
+          <t>ACS11202610291U00015</t>
+        </is>
+      </c>
+      <c r="E240" s="6" t="inlineStr">
+        <is>
+          <t>SW_LH_8P</t>
+        </is>
+      </c>
+      <c r="F240" s="7" t="inlineStr">
+        <is>
+          <t>BP00000129:ACS11202610291U00015</t>
+        </is>
+      </c>
+      <c r="G240" s="6" t="inlineStr"/>
+      <c r="H240" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
zpl code updated and qr size problem is still there
</commit_message>
<xml_diff>
--- a/models/hv/data/pack_id_scan_log.xlsx
+++ b/models/hv/data/pack_id_scan_log.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3036" yWindow="2340" windowWidth="11268" windowHeight="9900" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Pack ID" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pack ID" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H240"/>
+  <dimension ref="A1:H250"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4" outlineLevelCol="0"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -8119,6 +8119,326 @@
       <c r="G240" s="6" t="inlineStr"/>
       <c r="H240" s="6" t="inlineStr"/>
     </row>
+    <row r="241" ht="18" customHeight="1">
+      <c r="A241" s="4" t="n">
+        <v>240</v>
+      </c>
+      <c r="B241" s="4" t="inlineStr">
+        <is>
+          <t>30 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C241" s="4" t="inlineStr">
+        <is>
+          <t>09:21:04 AM</t>
+        </is>
+      </c>
+      <c r="D241" s="5" t="inlineStr">
+        <is>
+          <t>ACS21202610301R00001</t>
+        </is>
+      </c>
+      <c r="E241" s="4" t="inlineStr">
+        <is>
+          <t>SW_RH_8P</t>
+        </is>
+      </c>
+      <c r="F241" s="5" t="inlineStr">
+        <is>
+          <t>BP00000129:ACS21202610301R00001</t>
+        </is>
+      </c>
+      <c r="G241" s="4" t="inlineStr"/>
+      <c r="H241" s="4" t="inlineStr"/>
+    </row>
+    <row r="242" ht="18" customHeight="1">
+      <c r="A242" s="6" t="n">
+        <v>241</v>
+      </c>
+      <c r="B242" s="6" t="inlineStr">
+        <is>
+          <t>30 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C242" s="6" t="inlineStr">
+        <is>
+          <t>09:21:12 AM</t>
+        </is>
+      </c>
+      <c r="D242" s="7" t="inlineStr">
+        <is>
+          <t>ACS11202610301R00001</t>
+        </is>
+      </c>
+      <c r="E242" s="6" t="inlineStr">
+        <is>
+          <t>SW_LH_8P</t>
+        </is>
+      </c>
+      <c r="F242" s="7" t="inlineStr">
+        <is>
+          <t>BP00000129:ACS11202610301R00001</t>
+        </is>
+      </c>
+      <c r="G242" s="6" t="inlineStr"/>
+      <c r="H242" s="6" t="inlineStr"/>
+    </row>
+    <row r="243" ht="18" customHeight="1">
+      <c r="A243" s="4" t="n">
+        <v>242</v>
+      </c>
+      <c r="B243" s="4" t="inlineStr">
+        <is>
+          <t>15 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C243" s="4" t="inlineStr">
+        <is>
+          <t>09:21:53 AM</t>
+        </is>
+      </c>
+      <c r="D243" s="5" t="inlineStr">
+        <is>
+          <t>ABA61202609151R00276</t>
+        </is>
+      </c>
+      <c r="E243" s="4" t="inlineStr">
+        <is>
+          <t>27P</t>
+        </is>
+      </c>
+      <c r="F243" s="5" t="inlineStr">
+        <is>
+          <t>VQ150030:ABA61202609151R00276</t>
+        </is>
+      </c>
+      <c r="G243" s="4" t="inlineStr"/>
+      <c r="H243" s="4" t="inlineStr"/>
+    </row>
+    <row r="244" ht="18" customHeight="1">
+      <c r="A244" s="6" t="n">
+        <v>243</v>
+      </c>
+      <c r="B244" s="6" t="inlineStr">
+        <is>
+          <t>24 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C244" s="6" t="inlineStr">
+        <is>
+          <t>09:26:48 AM</t>
+        </is>
+      </c>
+      <c r="D244" s="7" t="inlineStr">
+        <is>
+          <t>ABA31202609241R00295</t>
+        </is>
+      </c>
+      <c r="E244" s="6" t="inlineStr">
+        <is>
+          <t>12P</t>
+        </is>
+      </c>
+      <c r="F244" s="7" t="inlineStr">
+        <is>
+          <t>VQ150000:ABA31202609241R00295</t>
+        </is>
+      </c>
+      <c r="G244" s="6" t="inlineStr"/>
+      <c r="H244" s="6" t="inlineStr"/>
+    </row>
+    <row r="245" ht="18" customHeight="1">
+      <c r="A245" s="4" t="n">
+        <v>244</v>
+      </c>
+      <c r="B245" s="4" t="inlineStr">
+        <is>
+          <t>24 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C245" s="4" t="inlineStr">
+        <is>
+          <t>09:27:54 AM</t>
+        </is>
+      </c>
+      <c r="D245" s="5" t="inlineStr">
+        <is>
+          <t>ABA31202609241R00295</t>
+        </is>
+      </c>
+      <c r="E245" s="4" t="inlineStr">
+        <is>
+          <t>12P</t>
+        </is>
+      </c>
+      <c r="F245" s="5" t="inlineStr">
+        <is>
+          <t>VQ150000:ABA31202609241R00295</t>
+        </is>
+      </c>
+      <c r="G245" s="4" t="inlineStr"/>
+      <c r="H245" s="4" t="inlineStr"/>
+    </row>
+    <row r="246" ht="18" customHeight="1">
+      <c r="A246" s="6" t="n">
+        <v>245</v>
+      </c>
+      <c r="B246" s="6" t="inlineStr">
+        <is>
+          <t>30 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C246" s="6" t="inlineStr">
+        <is>
+          <t>09:31:36 AM</t>
+        </is>
+      </c>
+      <c r="D246" s="7" t="inlineStr">
+        <is>
+          <t>ACS31202610301R00002</t>
+        </is>
+      </c>
+      <c r="E246" s="6" t="inlineStr">
+        <is>
+          <t>SW_LH_10P</t>
+        </is>
+      </c>
+      <c r="F246" s="7" t="inlineStr">
+        <is>
+          <t>BP00000002:ACS31202610301R00002</t>
+        </is>
+      </c>
+      <c r="G246" s="6" t="inlineStr"/>
+      <c r="H246" s="6" t="inlineStr"/>
+    </row>
+    <row r="247" ht="18" customHeight="1">
+      <c r="A247" s="4" t="n">
+        <v>246</v>
+      </c>
+      <c r="B247" s="4" t="inlineStr">
+        <is>
+          <t>30 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C247" s="4" t="inlineStr">
+        <is>
+          <t>10:22:49 AM</t>
+        </is>
+      </c>
+      <c r="D247" s="5" t="inlineStr">
+        <is>
+          <t>ABA51202610301U00005</t>
+        </is>
+      </c>
+      <c r="E247" s="4" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F247" s="5" t="inlineStr">
+        <is>
+          <t>VX156060:ABA51202610301U00005</t>
+        </is>
+      </c>
+      <c r="G247" s="4" t="inlineStr"/>
+      <c r="H247" s="4" t="inlineStr"/>
+    </row>
+    <row r="248" ht="18" customHeight="1">
+      <c r="A248" s="6" t="n">
+        <v>247</v>
+      </c>
+      <c r="B248" s="6" t="inlineStr">
+        <is>
+          <t>30 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C248" s="6" t="inlineStr">
+        <is>
+          <t>10:22:54 AM</t>
+        </is>
+      </c>
+      <c r="D248" s="7" t="inlineStr">
+        <is>
+          <t>ABA51202610301R00006</t>
+        </is>
+      </c>
+      <c r="E248" s="6" t="inlineStr">
+        <is>
+          <t>24P</t>
+        </is>
+      </c>
+      <c r="F248" s="7" t="inlineStr">
+        <is>
+          <t>VQ150020:ABA51202610301R00006</t>
+        </is>
+      </c>
+      <c r="G248" s="6" t="inlineStr"/>
+      <c r="H248" s="6" t="inlineStr"/>
+    </row>
+    <row r="249" ht="18" customHeight="1">
+      <c r="A249" s="4" t="n">
+        <v>248</v>
+      </c>
+      <c r="B249" s="4" t="inlineStr">
+        <is>
+          <t>30 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C249" s="4" t="inlineStr">
+        <is>
+          <t>10:22:59 AM</t>
+        </is>
+      </c>
+      <c r="D249" s="5" t="inlineStr">
+        <is>
+          <t>ACS11202610301R00007</t>
+        </is>
+      </c>
+      <c r="E249" s="4" t="inlineStr">
+        <is>
+          <t>SW_LH_8P</t>
+        </is>
+      </c>
+      <c r="F249" s="5" t="inlineStr">
+        <is>
+          <t>BP00000129:ACS11202610301R00007</t>
+        </is>
+      </c>
+      <c r="G249" s="4" t="inlineStr"/>
+      <c r="H249" s="4" t="inlineStr"/>
+    </row>
+    <row r="250" ht="18" customHeight="1">
+      <c r="A250" s="6" t="n">
+        <v>249</v>
+      </c>
+      <c r="B250" s="6" t="inlineStr">
+        <is>
+          <t>30 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C250" s="6" t="inlineStr">
+        <is>
+          <t>10:23:04 AM</t>
+        </is>
+      </c>
+      <c r="D250" s="7" t="inlineStr">
+        <is>
+          <t>ADT11202610301R00008</t>
+        </is>
+      </c>
+      <c r="E250" s="6" t="inlineStr">
+        <is>
+          <t>TS_8P</t>
+        </is>
+      </c>
+      <c r="F250" s="7" t="inlineStr">
+        <is>
+          <t>BP00000131:ADT11202610301R00008</t>
+        </is>
+      </c>
+      <c r="G250" s="6" t="inlineStr"/>
+      <c r="H250" s="6" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>